<commit_message>
Add robot control settings and full-work handling
</commit_message>
<xml_diff>
--- a/Tín hiệu Robot Nittan.xlsx
+++ b/Tín hiệu Robot Nittan.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Nittan\WpfCompanyApp_net58\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426CAE63-15AB-44DF-9349-4DE8F481E9E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13716" windowHeight="7152"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="107">
   <si>
     <t>x</t>
   </si>
@@ -47,12 +48,6 @@
     <t>DI5</t>
   </si>
   <si>
-    <t>DI6</t>
-  </si>
-  <si>
-    <t>DI7</t>
-  </si>
-  <si>
     <t>XL1_Down</t>
   </si>
   <si>
@@ -95,9 +90,6 @@
     <t>CI3</t>
   </si>
   <si>
-    <t>CI4</t>
-  </si>
-  <si>
     <t>CI5</t>
   </si>
   <si>
@@ -119,12 +111,6 @@
     <t>Door2</t>
   </si>
   <si>
-    <t>Full</t>
-  </si>
-  <si>
-    <t>Stop</t>
-  </si>
-  <si>
     <t>Reset</t>
   </si>
   <si>
@@ -137,9 +123,6 @@
     <t>Cảm biến cửa 2</t>
   </si>
   <si>
-    <t>tín hiệu van đã đầy</t>
-  </si>
-  <si>
     <t>nút nhấn</t>
   </si>
   <si>
@@ -296,24 +279,6 @@
     <t>Cảm biến trên XL3</t>
   </si>
   <si>
-    <t>Remote IO</t>
-  </si>
-  <si>
-    <t>DI8</t>
-  </si>
-  <si>
-    <t>ss1</t>
-  </si>
-  <si>
-    <t>ss2</t>
-  </si>
-  <si>
-    <t>ss3</t>
-  </si>
-  <si>
-    <t>Cảm biến áp suất khí</t>
-  </si>
-  <si>
     <t>Cảm biến Basket 1</t>
   </si>
   <si>
@@ -321,19 +286,97 @@
   </si>
   <si>
     <t>Sub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X5 </t>
+  </si>
+  <si>
+    <t>X6</t>
+  </si>
+  <si>
+    <t>X7</t>
+  </si>
+  <si>
+    <t>Door3</t>
+  </si>
+  <si>
+    <t>Door4</t>
+  </si>
+  <si>
+    <t>Cảm biến cửa 3</t>
+  </si>
+  <si>
+    <t>Cảm biến cửa 4</t>
+  </si>
+  <si>
+    <t>X0</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>X3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X4 </t>
+  </si>
+  <si>
+    <t>Cảm biến áp xuất tổng</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 1</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 2</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 3</t>
+  </si>
+  <si>
+    <t>plc</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> cảm biến Máy1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> cảm biến Máy2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF081B3A"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFA31515"/>
+      <name val="Cascadia Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -408,10 +451,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -423,6 +465,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -703,405 +750,475 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:H34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="4" t="s">
-        <v>41</v>
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>8</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="4" t="s">
-        <v>43</v>
+        <v>9</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="4" t="s">
-        <v>44</v>
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="4" t="s">
-        <v>45</v>
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="4" t="s">
-        <v>48</v>
+      <c r="E10" s="4"/>
+      <c r="F10" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="3" t="s">
+      <c r="C15" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="4" t="s">
+      <c r="D17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="G14" s="1" t="s">
+      <c r="G18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="1" t="s">
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="5"/>
-      <c r="F17" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B18" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="5"/>
-      <c r="F18" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B19" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="4" t="s">
-        <v>67</v>
+      <c r="D19" s="2"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="G19" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B27" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="10">
+        <v>20480</v>
+      </c>
+      <c r="D27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28">
+        <v>20481</v>
+      </c>
+      <c r="D28" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>96</v>
+      </c>
+      <c r="C29" s="10">
+        <v>20482</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>97</v>
+      </c>
+      <c r="C30">
+        <v>20483</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
         <v>98</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B25" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>95</v>
+      <c r="C31" s="10">
+        <v>20484</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32">
+        <v>20485</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="10">
+        <v>20486</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34">
+        <v>20487</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1110,6 +1227,7 @@
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="B22:D22"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update robot I/O mapping and enforce safe control states
</commit_message>
<xml_diff>
--- a/Tín hiệu Robot Nittan.xlsx
+++ b/Tín hiệu Robot Nittan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Nittan\WpfCompanyApp_net58\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426CAE63-15AB-44DF-9349-4DE8F481E9E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8331F27E-9F63-42C6-B944-0CE67774374A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="107">
-  <si>
-    <t>x</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="98">
   <si>
     <t>DI0</t>
   </si>
@@ -66,18 +63,6 @@
     <t>XL3_Up</t>
   </si>
   <si>
-    <t>SS_SC1</t>
-  </si>
-  <si>
-    <t>SS_SC2</t>
-  </si>
-  <si>
-    <t>Cảm biến khí âm XL1</t>
-  </si>
-  <si>
-    <t>Cảm biến khí âm XL2</t>
-  </si>
-  <si>
     <t>CI0</t>
   </si>
   <si>
@@ -96,15 +81,6 @@
     <t>CI6</t>
   </si>
   <si>
-    <t>CI7</t>
-  </si>
-  <si>
-    <t>SS_SC3</t>
-  </si>
-  <si>
-    <t>Cảm biến khí âm XL3</t>
-  </si>
-  <si>
     <t>Door1</t>
   </si>
   <si>
@@ -123,9 +99,6 @@
     <t>Cảm biến cửa 2</t>
   </si>
   <si>
-    <t>nút nhấn</t>
-  </si>
-  <si>
     <t>INPUT</t>
   </si>
   <si>
@@ -177,15 +150,6 @@
     <t>Trigger camera</t>
   </si>
   <si>
-    <t>Núm hút XL1</t>
-  </si>
-  <si>
-    <t>Núm hút XL2</t>
-  </si>
-  <si>
-    <t>Núm hút XL3</t>
-  </si>
-  <si>
     <t>Trigger</t>
   </si>
   <si>
@@ -210,9 +174,6 @@
     <t>CO6</t>
   </si>
   <si>
-    <t>CO7</t>
-  </si>
-  <si>
     <t>Red</t>
   </si>
   <si>
@@ -231,15 +192,6 @@
     <t>còi</t>
   </si>
   <si>
-    <t>van thổi xilanh 1</t>
-  </si>
-  <si>
-    <t>van thổi xilanh 2</t>
-  </si>
-  <si>
-    <t>van thổi xilanh 3</t>
-  </si>
-  <si>
     <t>Blow1</t>
   </si>
   <si>
@@ -249,48 +201,12 @@
     <t>Blow3</t>
   </si>
   <si>
-    <t>van hút phụ</t>
-  </si>
-  <si>
-    <t>Điều khiển XL1</t>
-  </si>
-  <si>
-    <t>Điều khiển XL2</t>
-  </si>
-  <si>
-    <t>Điều khiển XL3</t>
-  </si>
-  <si>
-    <t>Cảm biến dưới XL1</t>
-  </si>
-  <si>
-    <t>Cảm biến dưới XL2</t>
-  </si>
-  <si>
-    <t>Cảm biến dưới XL3</t>
-  </si>
-  <si>
-    <t>Cảm biến trên XL2</t>
-  </si>
-  <si>
-    <t>Cảm biến trên XL1</t>
-  </si>
-  <si>
-    <t>Cảm biến trên XL3</t>
-  </si>
-  <si>
     <t>Cảm biến Basket 1</t>
   </si>
   <si>
     <t>Cảm biến Basket 2</t>
   </si>
   <si>
-    <t>Sub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">X5 </t>
-  </si>
-  <si>
     <t>X6</t>
   </si>
   <si>
@@ -330,15 +246,6 @@
     <t>X5</t>
   </si>
   <si>
-    <t>Cảm biến hút đươc sản phẩm 1</t>
-  </si>
-  <si>
-    <t>Cảm biến hút đươc sản phẩm 2</t>
-  </si>
-  <si>
-    <t>Cảm biến hút đươc sản phẩm 3</t>
-  </si>
-  <si>
     <t>plc</t>
   </si>
   <si>
@@ -346,6 +253,72 @@
   </si>
   <si>
     <t xml:space="preserve"> cảm biến Máy2</t>
+  </si>
+  <si>
+    <t>CI4</t>
+  </si>
+  <si>
+    <t>Stop</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 1 của đầu tool1(XL1)</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 2 của đầu tool2(XL2)</t>
+  </si>
+  <si>
+    <t>Cảm biến hút đươc sản phẩm 3 của đầu tool3(XL3)</t>
+  </si>
+  <si>
+    <t>van thổi khí đầu tool1(XL1)</t>
+  </si>
+  <si>
+    <t>van thổi khí đầu tool3(XL3)</t>
+  </si>
+  <si>
+    <t>van thổi khí đầu tool2(XL2)</t>
+  </si>
+  <si>
+    <t>Núm hút đầu tool1 (XL1)</t>
+  </si>
+  <si>
+    <t>Núm hút đầu tool2 (XL2)</t>
+  </si>
+  <si>
+    <t>Núm hút đầu tool3 (XL3)</t>
+  </si>
+  <si>
+    <t>Điều khiển XL3( đầu tool3)</t>
+  </si>
+  <si>
+    <t>Điều khiển XL2 (đầu tool2)</t>
+  </si>
+  <si>
+    <t>Điều khiển XL1(đầu tool1)</t>
+  </si>
+  <si>
+    <t>Cảm biến dưới XL1(đầu tool1)</t>
+  </si>
+  <si>
+    <t>Cảm biến trên XL1(đầu tool1)</t>
+  </si>
+  <si>
+    <t>Cảm biến dưới XL2(đầu tool2)</t>
+  </si>
+  <si>
+    <t>Cảm biến trên XL2(đầu tool2)</t>
+  </si>
+  <si>
+    <t>Cảm biến dưới XL3(đầu tool3)</t>
+  </si>
+  <si>
+    <t>Cảm biến trên XL3(đầu tool3)</t>
+  </si>
+  <si>
+    <t>nút nhấn  (phần cứng)</t>
+  </si>
+  <si>
+    <t>nút nhấn (phần cứng)</t>
   </si>
 </sst>
 </file>
@@ -451,12 +424,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -465,11 +442,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -754,184 +726,172 @@
   <dimension ref="B2:H34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33" customWidth="1"/>
+    <col min="4" max="4" width="44.42578125" customWidth="1"/>
+    <col min="8" max="8" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="6"/>
+      <c r="B2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="F2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="3" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="3" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>50</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="3" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>51</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="3" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="2"/>
       <c r="E9" s="4"/>
       <c r="F9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="H9" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="2"/>
       <c r="E10" s="4"/>
       <c r="F10" s="3" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -940,175 +900,170 @@
       <c r="E11" s="4"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="2"/>
       <c r="E12" s="4"/>
       <c r="F12" s="3" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="3" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="3" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="D17" s="2" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="3" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="3" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="E19" s="4"/>
-      <c r="F19" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>74</v>
-      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
@@ -1127,98 +1082,98 @@
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>104</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="B27" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C27" s="10">
+      <c r="B27" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="6">
         <v>20480</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="C28">
         <v>20481</v>
       </c>
       <c r="D28" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>96</v>
-      </c>
-      <c r="C29" s="10">
+        <v>68</v>
+      </c>
+      <c r="C29" s="6">
         <v>20482</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="C30">
         <v>20483</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>98</v>
-      </c>
-      <c r="C31" s="10">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6">
         <v>20484</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>99</v>
+      <c r="D31" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="C32">
         <v>20485</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>101</v>
+      <c r="D32" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="10">
+        <v>60</v>
+      </c>
+      <c r="C33" s="6">
         <v>20486</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>102</v>
+      <c r="D33" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="C34">
         <v>20487</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>103</v>
+      <c r="D34" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>